<commit_message>
feat: add CEADS parser and refresh coverage docs
</commit_message>
<xml_diff>
--- a/doc/source/_static/data/Country_coverage.xlsx
+++ b/doc/source/_static/data/Country_coverage.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Library/CloudStorage/OneDrive-SharedLibraries-PolitecnicodiMilano/DENG-SESAM - Documenti/c-Research/b-Models/MARIO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Documents/GitHub/MARIO/doc/source/_static/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E129C0C8-47F9-E647-B826-E27316F46B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45A92064-5E34-A543-B306-B24FE657FA07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17660" xr2:uid="{111A99A5-59A2-464B-993C-8B91581EF7C3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17660" activeTab="1" xr2:uid="{111A99A5-59A2-464B-993C-8B91581EF7C3}"/>
   </bookViews>
   <sheets>
     <sheet name="coverage" sheetId="1" r:id="rId1"/>
     <sheet name="concordance" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">concordance!$A$2:$L$259</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">concordance!$A$2:$N$259</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22642" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23192" uniqueCount="497">
   <si>
     <t>ABW</t>
   </si>
@@ -1430,6 +1430,108 @@
   <si>
     <t>0.60</t>
   </si>
+  <si>
+    <t>EUROSTAT</t>
+  </si>
+  <si>
+    <t>parse_eurostat</t>
+  </si>
+  <si>
+    <t>XK</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2015, 2016, 2017, 2018, 2019, 2020, 2021, 2022, 2023</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2015, 2016, 2017, 2018, 2019, 2020, 2021, 2022</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2018, 2019</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2015, 2016, 2017, 2018, 2019, 2020, 2021, 2022, 2023, 2024</t>
+  </si>
+  <si>
+    <t>2013, 2014, 2015, 2016, 2017, 2018</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2013, 2014, 2015, 2016, 2017, 2018, 2019, 2020, 2021, 2022</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2013, 2014, 2015, 2016, 2017, 2018, 2019, 2020</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2015, 2016, 2017, 2018, 2019, 2020, 2021, 2023</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2015, 2016, 2017, 2018</t>
+  </si>
+  <si>
+    <t>2013, 2014, 2015, 2016, 2017, 2018, 2019</t>
+  </si>
+  <si>
+    <t>2010, 2015, 2020</t>
+  </si>
+  <si>
+    <t>2010, 2015, 2020, 2022</t>
+  </si>
+  <si>
+    <t>2010, 2013, 2015, 2018, 2020, 2022</t>
+  </si>
+  <si>
+    <t>2010, 2015, 2016, 2020, 2021</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2015, 2016, 2017, 2018, 2019, 2020, 2021</t>
+  </si>
+  <si>
+    <t>2010, 2015, 2020, 2021, 2022, 2023</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2015, 2020</t>
+  </si>
+  <si>
+    <t>2010, 2015, 2016, 2017, 2018, 2019, 2020, 2021, 2022</t>
+  </si>
+  <si>
+    <t>2013, 2014, 2015, 2020</t>
+  </si>
+  <si>
+    <t>2010, 2013, 2015, 2017, 2020</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2015, 2016, 2017, 2018, 2019, 2021, 2022, 2023</t>
+  </si>
+  <si>
+    <t>2010, 2014, 2015, 2020</t>
+  </si>
+  <si>
+    <t>2012, 2015, 2023</t>
+  </si>
+  <si>
+    <t>2010, 2015, 2017</t>
+  </si>
+  <si>
+    <t>2015, 2019, 2020, 2022</t>
+  </si>
+  <si>
+    <t>2010, 2013, 2014, 2015, 2020</t>
+  </si>
+  <si>
+    <t>2010, 2014, 2015, 2016, 2017, 2018, 2020, 2022, 2023</t>
+  </si>
+  <si>
+    <t>2010, 2011, 2012, 2013, 2014, 2015, 2020</t>
+  </si>
+  <si>
+    <t>CEADS</t>
+  </si>
+  <si>
+    <t>parse_ceads</t>
+  </si>
+  <si>
+    <t>2018, 2020</t>
+  </si>
 </sst>
 </file>
 
@@ -1843,7 +1945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637C923A-C55A-2E43-A14B-2765261D910F}">
-  <dimension ref="A1:IR869"/>
+  <dimension ref="A1:IR948"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -1853,6 +1955,7 @@
     <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.5" customWidth="1"/>
     <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="51" width="6.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:252" x14ac:dyDescent="0.2">
@@ -69394,6 +69497,1718 @@
       </c>
       <c r="H869" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="870" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A870" t="s">
+        <v>463</v>
+      </c>
+      <c r="B870" t="s">
+        <v>464</v>
+      </c>
+      <c r="C870" t="s">
+        <v>344</v>
+      </c>
+      <c r="D870" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G870" t="s">
+        <v>289</v>
+      </c>
+      <c r="H870" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="871" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A871" t="s">
+        <v>463</v>
+      </c>
+      <c r="B871" t="s">
+        <v>464</v>
+      </c>
+      <c r="C871" t="s">
+        <v>344</v>
+      </c>
+      <c r="D871" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G871" t="s">
+        <v>289</v>
+      </c>
+      <c r="H871" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="872" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A872" t="s">
+        <v>463</v>
+      </c>
+      <c r="B872" t="s">
+        <v>464</v>
+      </c>
+      <c r="C872" t="s">
+        <v>344</v>
+      </c>
+      <c r="D872" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G872" t="s">
+        <v>289</v>
+      </c>
+      <c r="H872" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="873" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A873" t="s">
+        <v>463</v>
+      </c>
+      <c r="B873" t="s">
+        <v>464</v>
+      </c>
+      <c r="C873" t="s">
+        <v>344</v>
+      </c>
+      <c r="D873" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="G873" t="s">
+        <v>289</v>
+      </c>
+      <c r="H873" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="874" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A874" t="s">
+        <v>463</v>
+      </c>
+      <c r="B874" t="s">
+        <v>464</v>
+      </c>
+      <c r="C874" t="s">
+        <v>344</v>
+      </c>
+      <c r="D874" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G874" t="s">
+        <v>289</v>
+      </c>
+      <c r="H874" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="875" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A875" t="s">
+        <v>463</v>
+      </c>
+      <c r="B875" t="s">
+        <v>464</v>
+      </c>
+      <c r="C875" t="s">
+        <v>344</v>
+      </c>
+      <c r="D875" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="G875" t="s">
+        <v>289</v>
+      </c>
+      <c r="H875" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="876" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A876" t="s">
+        <v>463</v>
+      </c>
+      <c r="B876" t="s">
+        <v>464</v>
+      </c>
+      <c r="C876" t="s">
+        <v>344</v>
+      </c>
+      <c r="D876" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G876" t="s">
+        <v>289</v>
+      </c>
+      <c r="H876" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="877" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A877" t="s">
+        <v>463</v>
+      </c>
+      <c r="B877" t="s">
+        <v>464</v>
+      </c>
+      <c r="C877" t="s">
+        <v>344</v>
+      </c>
+      <c r="D877" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G877" t="s">
+        <v>289</v>
+      </c>
+      <c r="H877" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="878" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A878" t="s">
+        <v>463</v>
+      </c>
+      <c r="B878" t="s">
+        <v>464</v>
+      </c>
+      <c r="C878" t="s">
+        <v>344</v>
+      </c>
+      <c r="D878" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G878" t="s">
+        <v>289</v>
+      </c>
+      <c r="H878" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="879" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A879" t="s">
+        <v>463</v>
+      </c>
+      <c r="B879" t="s">
+        <v>464</v>
+      </c>
+      <c r="C879" t="s">
+        <v>344</v>
+      </c>
+      <c r="D879" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G879" t="s">
+        <v>289</v>
+      </c>
+      <c r="H879" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="880" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A880" t="s">
+        <v>463</v>
+      </c>
+      <c r="B880" t="s">
+        <v>464</v>
+      </c>
+      <c r="C880" t="s">
+        <v>344</v>
+      </c>
+      <c r="D880" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G880" t="s">
+        <v>289</v>
+      </c>
+      <c r="H880" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="881" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A881" t="s">
+        <v>463</v>
+      </c>
+      <c r="B881" t="s">
+        <v>464</v>
+      </c>
+      <c r="C881" t="s">
+        <v>344</v>
+      </c>
+      <c r="D881" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G881" t="s">
+        <v>289</v>
+      </c>
+      <c r="H881" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="882" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A882" t="s">
+        <v>463</v>
+      </c>
+      <c r="B882" t="s">
+        <v>464</v>
+      </c>
+      <c r="C882" t="s">
+        <v>344</v>
+      </c>
+      <c r="D882" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G882" t="s">
+        <v>289</v>
+      </c>
+      <c r="H882" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="883" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A883" t="s">
+        <v>463</v>
+      </c>
+      <c r="B883" t="s">
+        <v>464</v>
+      </c>
+      <c r="C883" t="s">
+        <v>344</v>
+      </c>
+      <c r="D883" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G883" t="s">
+        <v>289</v>
+      </c>
+      <c r="H883" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="884" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A884" t="s">
+        <v>463</v>
+      </c>
+      <c r="B884" t="s">
+        <v>464</v>
+      </c>
+      <c r="C884" t="s">
+        <v>344</v>
+      </c>
+      <c r="D884" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G884" t="s">
+        <v>289</v>
+      </c>
+      <c r="H884" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="885" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A885" t="s">
+        <v>463</v>
+      </c>
+      <c r="B885" t="s">
+        <v>464</v>
+      </c>
+      <c r="C885" t="s">
+        <v>344</v>
+      </c>
+      <c r="D885" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G885" t="s">
+        <v>289</v>
+      </c>
+      <c r="H885" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="886" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A886" t="s">
+        <v>463</v>
+      </c>
+      <c r="B886" t="s">
+        <v>464</v>
+      </c>
+      <c r="C886" t="s">
+        <v>344</v>
+      </c>
+      <c r="D886" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G886" t="s">
+        <v>289</v>
+      </c>
+      <c r="H886" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="887" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A887" t="s">
+        <v>463</v>
+      </c>
+      <c r="B887" t="s">
+        <v>464</v>
+      </c>
+      <c r="C887" t="s">
+        <v>344</v>
+      </c>
+      <c r="D887" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G887" t="s">
+        <v>289</v>
+      </c>
+      <c r="H887" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="888" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A888" t="s">
+        <v>463</v>
+      </c>
+      <c r="B888" t="s">
+        <v>464</v>
+      </c>
+      <c r="C888" t="s">
+        <v>344</v>
+      </c>
+      <c r="D888" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G888" t="s">
+        <v>289</v>
+      </c>
+      <c r="H888" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="889" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A889" t="s">
+        <v>463</v>
+      </c>
+      <c r="B889" t="s">
+        <v>464</v>
+      </c>
+      <c r="C889" t="s">
+        <v>344</v>
+      </c>
+      <c r="D889" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G889" t="s">
+        <v>289</v>
+      </c>
+      <c r="H889" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="890" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A890" t="s">
+        <v>463</v>
+      </c>
+      <c r="B890" t="s">
+        <v>464</v>
+      </c>
+      <c r="C890" t="s">
+        <v>344</v>
+      </c>
+      <c r="D890" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="G890" t="s">
+        <v>289</v>
+      </c>
+      <c r="H890" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="891" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A891" t="s">
+        <v>463</v>
+      </c>
+      <c r="B891" t="s">
+        <v>464</v>
+      </c>
+      <c r="C891" t="s">
+        <v>344</v>
+      </c>
+      <c r="D891" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="G891" t="s">
+        <v>289</v>
+      </c>
+      <c r="H891" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="892" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A892" t="s">
+        <v>463</v>
+      </c>
+      <c r="B892" t="s">
+        <v>464</v>
+      </c>
+      <c r="C892" t="s">
+        <v>344</v>
+      </c>
+      <c r="D892" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="G892" t="s">
+        <v>289</v>
+      </c>
+      <c r="H892" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="893" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A893" t="s">
+        <v>463</v>
+      </c>
+      <c r="B893" t="s">
+        <v>464</v>
+      </c>
+      <c r="C893" t="s">
+        <v>344</v>
+      </c>
+      <c r="D893" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G893" t="s">
+        <v>289</v>
+      </c>
+      <c r="H893" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="894" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A894" t="s">
+        <v>463</v>
+      </c>
+      <c r="B894" t="s">
+        <v>464</v>
+      </c>
+      <c r="C894" t="s">
+        <v>344</v>
+      </c>
+      <c r="D894" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G894" t="s">
+        <v>289</v>
+      </c>
+      <c r="H894" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="895" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A895" t="s">
+        <v>463</v>
+      </c>
+      <c r="B895" t="s">
+        <v>464</v>
+      </c>
+      <c r="C895" t="s">
+        <v>344</v>
+      </c>
+      <c r="D895" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G895" t="s">
+        <v>289</v>
+      </c>
+      <c r="H895" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="896" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A896" t="s">
+        <v>463</v>
+      </c>
+      <c r="B896" t="s">
+        <v>464</v>
+      </c>
+      <c r="C896" t="s">
+        <v>344</v>
+      </c>
+      <c r="D896" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G896" t="s">
+        <v>289</v>
+      </c>
+      <c r="H896" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="897" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A897" t="s">
+        <v>463</v>
+      </c>
+      <c r="B897" t="s">
+        <v>464</v>
+      </c>
+      <c r="C897" t="s">
+        <v>344</v>
+      </c>
+      <c r="D897" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G897" t="s">
+        <v>289</v>
+      </c>
+      <c r="H897" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="898" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A898" t="s">
+        <v>463</v>
+      </c>
+      <c r="B898" t="s">
+        <v>464</v>
+      </c>
+      <c r="C898" t="s">
+        <v>344</v>
+      </c>
+      <c r="D898" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G898" t="s">
+        <v>289</v>
+      </c>
+      <c r="H898" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="899" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A899" t="s">
+        <v>463</v>
+      </c>
+      <c r="B899" t="s">
+        <v>464</v>
+      </c>
+      <c r="C899" t="s">
+        <v>344</v>
+      </c>
+      <c r="D899" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G899" t="s">
+        <v>289</v>
+      </c>
+      <c r="H899" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="900" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A900" t="s">
+        <v>463</v>
+      </c>
+      <c r="B900" t="s">
+        <v>464</v>
+      </c>
+      <c r="C900" t="s">
+        <v>344</v>
+      </c>
+      <c r="D900" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G900" t="s">
+        <v>289</v>
+      </c>
+      <c r="H900" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="901" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A901" t="s">
+        <v>463</v>
+      </c>
+      <c r="B901" t="s">
+        <v>464</v>
+      </c>
+      <c r="C901" t="s">
+        <v>344</v>
+      </c>
+      <c r="D901" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="G901" t="s">
+        <v>289</v>
+      </c>
+      <c r="H901" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="902" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A902" t="s">
+        <v>463</v>
+      </c>
+      <c r="B902" t="s">
+        <v>464</v>
+      </c>
+      <c r="C902" t="s">
+        <v>344</v>
+      </c>
+      <c r="D902" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="G902" t="s">
+        <v>289</v>
+      </c>
+      <c r="H902" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="903" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A903" t="s">
+        <v>463</v>
+      </c>
+      <c r="B903" t="s">
+        <v>464</v>
+      </c>
+      <c r="C903" t="s">
+        <v>344</v>
+      </c>
+      <c r="D903" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="G903" t="s">
+        <v>289</v>
+      </c>
+      <c r="H903" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="904" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A904" t="s">
+        <v>463</v>
+      </c>
+      <c r="B904" t="s">
+        <v>464</v>
+      </c>
+      <c r="C904" t="s">
+        <v>248</v>
+      </c>
+      <c r="D904" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="F904" t="s">
+        <v>338</v>
+      </c>
+      <c r="G904" t="s">
+        <v>289</v>
+      </c>
+      <c r="H904" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="905" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A905" t="s">
+        <v>463</v>
+      </c>
+      <c r="B905" t="s">
+        <v>464</v>
+      </c>
+      <c r="C905" t="s">
+        <v>248</v>
+      </c>
+      <c r="D905" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F905" t="s">
+        <v>338</v>
+      </c>
+      <c r="G905" t="s">
+        <v>289</v>
+      </c>
+      <c r="H905" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="906" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A906" t="s">
+        <v>463</v>
+      </c>
+      <c r="B906" t="s">
+        <v>464</v>
+      </c>
+      <c r="C906" t="s">
+        <v>248</v>
+      </c>
+      <c r="D906" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="F906" t="s">
+        <v>338</v>
+      </c>
+      <c r="G906" t="s">
+        <v>289</v>
+      </c>
+      <c r="H906" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="907" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A907" t="s">
+        <v>463</v>
+      </c>
+      <c r="B907" t="s">
+        <v>464</v>
+      </c>
+      <c r="C907" t="s">
+        <v>248</v>
+      </c>
+      <c r="D907" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="F907" t="s">
+        <v>338</v>
+      </c>
+      <c r="G907" t="s">
+        <v>289</v>
+      </c>
+      <c r="H907" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="908" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A908" t="s">
+        <v>463</v>
+      </c>
+      <c r="B908" t="s">
+        <v>464</v>
+      </c>
+      <c r="C908" t="s">
+        <v>248</v>
+      </c>
+      <c r="D908" s="5">
+        <v>2010</v>
+      </c>
+      <c r="F908" t="s">
+        <v>338</v>
+      </c>
+      <c r="G908" t="s">
+        <v>289</v>
+      </c>
+      <c r="H908" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="909" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A909" t="s">
+        <v>463</v>
+      </c>
+      <c r="B909" t="s">
+        <v>464</v>
+      </c>
+      <c r="C909" t="s">
+        <v>248</v>
+      </c>
+      <c r="D909" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="F909" t="s">
+        <v>338</v>
+      </c>
+      <c r="G909" t="s">
+        <v>289</v>
+      </c>
+      <c r="H909" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="910" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A910" t="s">
+        <v>463</v>
+      </c>
+      <c r="B910" t="s">
+        <v>464</v>
+      </c>
+      <c r="C910" t="s">
+        <v>248</v>
+      </c>
+      <c r="D910" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="F910" t="s">
+        <v>338</v>
+      </c>
+      <c r="G910" t="s">
+        <v>289</v>
+      </c>
+      <c r="H910" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="911" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A911" t="s">
+        <v>463</v>
+      </c>
+      <c r="B911" t="s">
+        <v>464</v>
+      </c>
+      <c r="C911" t="s">
+        <v>248</v>
+      </c>
+      <c r="D911" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="F911" t="s">
+        <v>338</v>
+      </c>
+      <c r="G911" t="s">
+        <v>289</v>
+      </c>
+      <c r="H911" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="912" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A912" t="s">
+        <v>463</v>
+      </c>
+      <c r="B912" t="s">
+        <v>464</v>
+      </c>
+      <c r="C912" t="s">
+        <v>248</v>
+      </c>
+      <c r="D912" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F912" t="s">
+        <v>338</v>
+      </c>
+      <c r="G912" t="s">
+        <v>289</v>
+      </c>
+      <c r="H912" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="913" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A913" t="s">
+        <v>463</v>
+      </c>
+      <c r="B913" t="s">
+        <v>464</v>
+      </c>
+      <c r="C913" t="s">
+        <v>248</v>
+      </c>
+      <c r="D913" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F913" t="s">
+        <v>338</v>
+      </c>
+      <c r="G913" t="s">
+        <v>289</v>
+      </c>
+      <c r="H913" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="914" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A914" t="s">
+        <v>463</v>
+      </c>
+      <c r="B914" t="s">
+        <v>464</v>
+      </c>
+      <c r="C914" t="s">
+        <v>248</v>
+      </c>
+      <c r="D914" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="F914" t="s">
+        <v>338</v>
+      </c>
+      <c r="G914" t="s">
+        <v>289</v>
+      </c>
+      <c r="H914" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="915" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A915" t="s">
+        <v>463</v>
+      </c>
+      <c r="B915" t="s">
+        <v>464</v>
+      </c>
+      <c r="C915" t="s">
+        <v>248</v>
+      </c>
+      <c r="D915" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="F915" t="s">
+        <v>338</v>
+      </c>
+      <c r="G915" t="s">
+        <v>289</v>
+      </c>
+      <c r="H915" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="916" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A916" t="s">
+        <v>463</v>
+      </c>
+      <c r="B916" t="s">
+        <v>464</v>
+      </c>
+      <c r="C916" t="s">
+        <v>248</v>
+      </c>
+      <c r="D916" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="F916" t="s">
+        <v>338</v>
+      </c>
+      <c r="G916" t="s">
+        <v>289</v>
+      </c>
+      <c r="H916" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="917" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A917" t="s">
+        <v>463</v>
+      </c>
+      <c r="B917" t="s">
+        <v>464</v>
+      </c>
+      <c r="C917" t="s">
+        <v>248</v>
+      </c>
+      <c r="D917" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="F917" t="s">
+        <v>338</v>
+      </c>
+      <c r="G917" t="s">
+        <v>289</v>
+      </c>
+      <c r="H917" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="918" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A918" t="s">
+        <v>463</v>
+      </c>
+      <c r="B918" t="s">
+        <v>464</v>
+      </c>
+      <c r="C918" t="s">
+        <v>248</v>
+      </c>
+      <c r="D918" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="F918" t="s">
+        <v>338</v>
+      </c>
+      <c r="G918" t="s">
+        <v>289</v>
+      </c>
+      <c r="H918" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="919" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A919" t="s">
+        <v>463</v>
+      </c>
+      <c r="B919" t="s">
+        <v>464</v>
+      </c>
+      <c r="C919" t="s">
+        <v>248</v>
+      </c>
+      <c r="D919" s="5" t="s">
+        <v>483</v>
+      </c>
+      <c r="F919" t="s">
+        <v>338</v>
+      </c>
+      <c r="G919" t="s">
+        <v>289</v>
+      </c>
+      <c r="H919" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="920" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A920" t="s">
+        <v>463</v>
+      </c>
+      <c r="B920" t="s">
+        <v>464</v>
+      </c>
+      <c r="C920" t="s">
+        <v>248</v>
+      </c>
+      <c r="D920" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F920" t="s">
+        <v>338</v>
+      </c>
+      <c r="G920" t="s">
+        <v>289</v>
+      </c>
+      <c r="H920" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="921" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A921" t="s">
+        <v>463</v>
+      </c>
+      <c r="B921" t="s">
+        <v>464</v>
+      </c>
+      <c r="C921" t="s">
+        <v>248</v>
+      </c>
+      <c r="D921" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="F921" t="s">
+        <v>338</v>
+      </c>
+      <c r="G921" t="s">
+        <v>289</v>
+      </c>
+      <c r="H921" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="922" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A922" t="s">
+        <v>463</v>
+      </c>
+      <c r="B922" t="s">
+        <v>464</v>
+      </c>
+      <c r="C922" t="s">
+        <v>248</v>
+      </c>
+      <c r="D922" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F922" t="s">
+        <v>338</v>
+      </c>
+      <c r="G922" t="s">
+        <v>289</v>
+      </c>
+      <c r="H922" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="923" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A923" t="s">
+        <v>463</v>
+      </c>
+      <c r="B923" t="s">
+        <v>464</v>
+      </c>
+      <c r="C923" t="s">
+        <v>248</v>
+      </c>
+      <c r="D923" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F923" t="s">
+        <v>338</v>
+      </c>
+      <c r="G923" t="s">
+        <v>289</v>
+      </c>
+      <c r="H923" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="924" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A924" t="s">
+        <v>463</v>
+      </c>
+      <c r="B924" t="s">
+        <v>464</v>
+      </c>
+      <c r="C924" t="s">
+        <v>248</v>
+      </c>
+      <c r="D924" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="F924" t="s">
+        <v>338</v>
+      </c>
+      <c r="G924" t="s">
+        <v>289</v>
+      </c>
+      <c r="H924" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="925" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A925" t="s">
+        <v>463</v>
+      </c>
+      <c r="B925" t="s">
+        <v>464</v>
+      </c>
+      <c r="C925" t="s">
+        <v>248</v>
+      </c>
+      <c r="D925" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F925" t="s">
+        <v>338</v>
+      </c>
+      <c r="G925" t="s">
+        <v>289</v>
+      </c>
+      <c r="H925" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="926" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A926" t="s">
+        <v>463</v>
+      </c>
+      <c r="B926" t="s">
+        <v>464</v>
+      </c>
+      <c r="C926" t="s">
+        <v>248</v>
+      </c>
+      <c r="D926" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="F926" t="s">
+        <v>338</v>
+      </c>
+      <c r="G926" t="s">
+        <v>289</v>
+      </c>
+      <c r="H926" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="927" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A927" t="s">
+        <v>463</v>
+      </c>
+      <c r="B927" t="s">
+        <v>464</v>
+      </c>
+      <c r="C927" t="s">
+        <v>248</v>
+      </c>
+      <c r="D927" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F927" t="s">
+        <v>338</v>
+      </c>
+      <c r="G927" t="s">
+        <v>289</v>
+      </c>
+      <c r="H927" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="928" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A928" t="s">
+        <v>463</v>
+      </c>
+      <c r="B928" t="s">
+        <v>464</v>
+      </c>
+      <c r="C928" t="s">
+        <v>248</v>
+      </c>
+      <c r="D928" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="F928" t="s">
+        <v>338</v>
+      </c>
+      <c r="G928" t="s">
+        <v>289</v>
+      </c>
+      <c r="H928" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="929" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A929" t="s">
+        <v>463</v>
+      </c>
+      <c r="B929" t="s">
+        <v>464</v>
+      </c>
+      <c r="C929" t="s">
+        <v>248</v>
+      </c>
+      <c r="D929" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="F929" t="s">
+        <v>338</v>
+      </c>
+      <c r="G929" t="s">
+        <v>289</v>
+      </c>
+      <c r="H929" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="930" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A930" t="s">
+        <v>463</v>
+      </c>
+      <c r="B930" t="s">
+        <v>464</v>
+      </c>
+      <c r="C930" t="s">
+        <v>248</v>
+      </c>
+      <c r="D930" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F930" t="s">
+        <v>338</v>
+      </c>
+      <c r="G930" t="s">
+        <v>289</v>
+      </c>
+      <c r="H930" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="931" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A931" t="s">
+        <v>463</v>
+      </c>
+      <c r="B931" t="s">
+        <v>464</v>
+      </c>
+      <c r="C931" t="s">
+        <v>248</v>
+      </c>
+      <c r="D931" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="F931" t="s">
+        <v>338</v>
+      </c>
+      <c r="G931" t="s">
+        <v>289</v>
+      </c>
+      <c r="H931" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="932" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A932" t="s">
+        <v>463</v>
+      </c>
+      <c r="B932" t="s">
+        <v>464</v>
+      </c>
+      <c r="C932" t="s">
+        <v>248</v>
+      </c>
+      <c r="D932" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="F932" t="s">
+        <v>338</v>
+      </c>
+      <c r="G932" t="s">
+        <v>289</v>
+      </c>
+      <c r="H932" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="933" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A933" t="s">
+        <v>463</v>
+      </c>
+      <c r="B933" t="s">
+        <v>464</v>
+      </c>
+      <c r="C933" t="s">
+        <v>248</v>
+      </c>
+      <c r="D933" s="5">
+        <v>2015</v>
+      </c>
+      <c r="F933" t="s">
+        <v>337</v>
+      </c>
+      <c r="G933" t="s">
+        <v>289</v>
+      </c>
+      <c r="H933" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="934" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A934" t="s">
+        <v>463</v>
+      </c>
+      <c r="B934" t="s">
+        <v>464</v>
+      </c>
+      <c r="C934" t="s">
+        <v>248</v>
+      </c>
+      <c r="D934" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F934" t="s">
+        <v>337</v>
+      </c>
+      <c r="G934" t="s">
+        <v>289</v>
+      </c>
+      <c r="H934" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="935" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A935" t="s">
+        <v>463</v>
+      </c>
+      <c r="B935" t="s">
+        <v>464</v>
+      </c>
+      <c r="C935" t="s">
+        <v>248</v>
+      </c>
+      <c r="D935" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="F935" t="s">
+        <v>337</v>
+      </c>
+      <c r="G935" t="s">
+        <v>289</v>
+      </c>
+      <c r="H935" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="936" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A936" t="s">
+        <v>463</v>
+      </c>
+      <c r="B936" t="s">
+        <v>464</v>
+      </c>
+      <c r="C936" t="s">
+        <v>248</v>
+      </c>
+      <c r="D936" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="F936" t="s">
+        <v>337</v>
+      </c>
+      <c r="G936" t="s">
+        <v>289</v>
+      </c>
+      <c r="H936" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="937" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A937" t="s">
+        <v>463</v>
+      </c>
+      <c r="B937" t="s">
+        <v>464</v>
+      </c>
+      <c r="C937" t="s">
+        <v>248</v>
+      </c>
+      <c r="D937" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="F937" t="s">
+        <v>337</v>
+      </c>
+      <c r="G937" t="s">
+        <v>289</v>
+      </c>
+      <c r="H937" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="938" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A938" t="s">
+        <v>463</v>
+      </c>
+      <c r="B938" t="s">
+        <v>464</v>
+      </c>
+      <c r="C938" t="s">
+        <v>248</v>
+      </c>
+      <c r="D938" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F938" t="s">
+        <v>337</v>
+      </c>
+      <c r="G938" t="s">
+        <v>289</v>
+      </c>
+      <c r="H938" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="939" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A939" t="s">
+        <v>463</v>
+      </c>
+      <c r="B939" t="s">
+        <v>464</v>
+      </c>
+      <c r="C939" t="s">
+        <v>248</v>
+      </c>
+      <c r="D939" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="F939" t="s">
+        <v>337</v>
+      </c>
+      <c r="G939" t="s">
+        <v>289</v>
+      </c>
+      <c r="H939" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="940" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A940" t="s">
+        <v>463</v>
+      </c>
+      <c r="B940" t="s">
+        <v>464</v>
+      </c>
+      <c r="C940" t="s">
+        <v>248</v>
+      </c>
+      <c r="D940" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="F940" t="s">
+        <v>337</v>
+      </c>
+      <c r="G940" t="s">
+        <v>289</v>
+      </c>
+      <c r="H940" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="941" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A941" t="s">
+        <v>463</v>
+      </c>
+      <c r="B941" t="s">
+        <v>464</v>
+      </c>
+      <c r="C941" t="s">
+        <v>248</v>
+      </c>
+      <c r="D941" s="5" t="s">
+        <v>483</v>
+      </c>
+      <c r="F941" t="s">
+        <v>337</v>
+      </c>
+      <c r="G941" t="s">
+        <v>289</v>
+      </c>
+      <c r="H941" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="942" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A942" t="s">
+        <v>463</v>
+      </c>
+      <c r="B942" t="s">
+        <v>464</v>
+      </c>
+      <c r="C942" t="s">
+        <v>248</v>
+      </c>
+      <c r="D942" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="F942" t="s">
+        <v>337</v>
+      </c>
+      <c r="G942" t="s">
+        <v>289</v>
+      </c>
+      <c r="H942" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="943" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A943" t="s">
+        <v>463</v>
+      </c>
+      <c r="B943" t="s">
+        <v>464</v>
+      </c>
+      <c r="C943" t="s">
+        <v>248</v>
+      </c>
+      <c r="D943" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="F943" t="s">
+        <v>337</v>
+      </c>
+      <c r="G943" t="s">
+        <v>289</v>
+      </c>
+      <c r="H943" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="944" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A944" t="s">
+        <v>463</v>
+      </c>
+      <c r="B944" t="s">
+        <v>464</v>
+      </c>
+      <c r="C944" t="s">
+        <v>248</v>
+      </c>
+      <c r="D944" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="F944" t="s">
+        <v>337</v>
+      </c>
+      <c r="G944" t="s">
+        <v>289</v>
+      </c>
+      <c r="H944" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="945" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A945" t="s">
+        <v>463</v>
+      </c>
+      <c r="B945" t="s">
+        <v>464</v>
+      </c>
+      <c r="C945" t="s">
+        <v>248</v>
+      </c>
+      <c r="D945" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="F945" t="s">
+        <v>337</v>
+      </c>
+      <c r="G945" t="s">
+        <v>289</v>
+      </c>
+      <c r="H945" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="946" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A946" t="s">
+        <v>463</v>
+      </c>
+      <c r="B946" t="s">
+        <v>464</v>
+      </c>
+      <c r="C946" t="s">
+        <v>248</v>
+      </c>
+      <c r="D946" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="F946" t="s">
+        <v>337</v>
+      </c>
+      <c r="G946" t="s">
+        <v>289</v>
+      </c>
+      <c r="H946" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="947" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A947" t="s">
+        <v>463</v>
+      </c>
+      <c r="B947" t="s">
+        <v>464</v>
+      </c>
+      <c r="C947" t="s">
+        <v>248</v>
+      </c>
+      <c r="D947" s="5">
+        <v>2015</v>
+      </c>
+      <c r="F947" t="s">
+        <v>337</v>
+      </c>
+      <c r="G947" t="s">
+        <v>289</v>
+      </c>
+      <c r="H947" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="948" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A948" t="s">
+        <v>494</v>
+      </c>
+      <c r="B948" t="s">
+        <v>495</v>
+      </c>
+      <c r="C948" t="s">
+        <v>248</v>
+      </c>
+      <c r="D948" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="G948" t="s">
+        <v>288</v>
+      </c>
+      <c r="H948" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -69403,19 +71218,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04039038-B78D-F44F-9F75-C547258D839A}">
-  <dimension ref="A1:M259"/>
+  <dimension ref="A1:O259"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>447</v>
       </c>
@@ -69447,16 +71263,22 @@
         <v>415</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -69472,8 +71294,9 @@
       <c r="J3" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K3" s="1"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -69491,8 +71314,9 @@
       <c r="J4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K4" s="1"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -69512,8 +71336,9 @@
       <c r="J5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>252</v>
       </c>
@@ -69524,8 +71349,9 @@
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>434</v>
       </c>
@@ -69533,8 +71359,9 @@
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K7" s="1"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -69557,8 +71384,11 @@
       <c r="J8" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K8" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -69572,8 +71402,9 @@
       <c r="J9" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>253</v>
       </c>
@@ -69587,8 +71418,9 @@
       <c r="J10" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -69610,8 +71442,9 @@
       <c r="J11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -69638,8 +71471,9 @@
       <c r="J12" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -69658,8 +71492,9 @@
       <c r="J13" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -69670,8 +71505,9 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K14" s="1"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>255</v>
       </c>
@@ -69682,8 +71518,9 @@
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K15" s="1"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>256</v>
       </c>
@@ -69694,8 +71531,9 @@
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K16" s="1"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -69709,8 +71547,9 @@
       <c r="J17" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K17" s="1"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -69739,8 +71578,9 @@
       <c r="J18" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K18" s="2"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -69768,8 +71608,11 @@
       <c r="J19" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K19" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -69783,12 +71626,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -69802,7 +71645,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -69830,8 +71673,11 @@
       <c r="J23" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K23" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>15</v>
       </c>
@@ -69845,7 +71691,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>254</v>
       </c>
@@ -69853,7 +71699,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>16</v>
       </c>
@@ -69867,7 +71713,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -69887,7 +71733,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -69915,8 +71761,11 @@
       <c r="J28" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K28" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>19</v>
       </c>
@@ -69930,7 +71779,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>20</v>
       </c>
@@ -69944,7 +71793,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -69958,7 +71807,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>257</v>
       </c>
@@ -69966,7 +71815,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>22</v>
       </c>
@@ -69983,7 +71832,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -69997,7 +71846,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>24</v>
       </c>
@@ -70008,7 +71857,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -70028,7 +71877,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>26</v>
       </c>
@@ -70060,7 +71909,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -70071,7 +71920,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>28</v>
       </c>
@@ -70091,7 +71940,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>29</v>
       </c>
@@ -70108,7 +71957,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>258</v>
       </c>
@@ -70116,7 +71965,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>30</v>
       </c>
@@ -70130,7 +71979,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>31</v>
       </c>
@@ -70144,7 +71993,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>32</v>
       </c>
@@ -70172,11 +72021,11 @@
       <c r="J44" t="s">
         <v>32</v>
       </c>
-      <c r="L44" t="s">
+      <c r="N44" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>259</v>
       </c>
@@ -70184,7 +72033,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>33</v>
       </c>
@@ -70213,12 +72062,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>34</v>
       </c>
@@ -70241,7 +72090,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>35</v>
       </c>
@@ -70269,8 +72118,11 @@
       <c r="J49" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M49" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>36</v>
       </c>
@@ -70287,7 +72139,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>37</v>
       </c>
@@ -70304,7 +72156,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>38</v>
       </c>
@@ -70321,7 +72173,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>39</v>
       </c>
@@ -70335,7 +72187,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>260</v>
       </c>
@@ -70343,7 +72195,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>40</v>
       </c>
@@ -70366,7 +72218,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>41</v>
       </c>
@@ -70374,7 +72226,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>42</v>
       </c>
@@ -70388,7 +72240,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>43</v>
       </c>
@@ -70408,7 +72260,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>44</v>
       </c>
@@ -70422,7 +72274,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>45</v>
       </c>
@@ -70430,7 +72282,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>261</v>
       </c>
@@ -70438,7 +72290,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>46</v>
       </c>
@@ -70449,7 +72301,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>47</v>
       </c>
@@ -70477,8 +72329,11 @@
       <c r="J63" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K63" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>48</v>
       </c>
@@ -70506,8 +72361,11 @@
       <c r="J64" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K64" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>49</v>
       </c>
@@ -70535,8 +72393,11 @@
       <c r="J65" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K65" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>50</v>
       </c>
@@ -70550,7 +72411,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>51</v>
       </c>
@@ -70558,7 +72419,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>52</v>
       </c>
@@ -70586,8 +72447,11 @@
       <c r="J68" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K68" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>53</v>
       </c>
@@ -70604,7 +72468,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>380</v>
       </c>
@@ -70612,7 +72476,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>54</v>
       </c>
@@ -70626,17 +72490,17 @@
         <v>54</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>55</v>
       </c>
@@ -70656,7 +72520,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>56</v>
       </c>
@@ -70676,7 +72540,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>57</v>
       </c>
@@ -70690,7 +72554,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>262</v>
       </c>
@@ -70698,7 +72562,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>58</v>
       </c>
@@ -70726,8 +72590,11 @@
       <c r="J78" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K78" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>59</v>
       </c>
@@ -70755,8 +72622,11 @@
       <c r="J79" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K79" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>60</v>
       </c>
@@ -70770,7 +72640,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>61</v>
       </c>
@@ -70798,8 +72668,11 @@
       <c r="J81" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K81" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>62</v>
       </c>
@@ -70813,7 +72686,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>263</v>
       </c>
@@ -70821,7 +72694,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>63</v>
       </c>
@@ -70849,8 +72722,11 @@
       <c r="J84" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K84" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>64</v>
       </c>
@@ -70858,7 +72734,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>65</v>
       </c>
@@ -70866,7 +72742,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>66</v>
       </c>
@@ -70880,7 +72756,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>67</v>
       </c>
@@ -70908,8 +72784,11 @@
       <c r="J88" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K88" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>68</v>
       </c>
@@ -70929,12 +72808,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>69</v>
       </c>
@@ -70948,7 +72827,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>70</v>
       </c>
@@ -70956,7 +72835,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>71</v>
       </c>
@@ -70970,7 +72849,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>264</v>
       </c>
@@ -70978,7 +72857,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>72</v>
       </c>
@@ -70992,7 +72871,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>73</v>
       </c>
@@ -71000,7 +72879,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>74</v>
       </c>
@@ -71011,7 +72890,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>75</v>
       </c>
@@ -71039,8 +72918,11 @@
       <c r="J98" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K98" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>76</v>
       </c>
@@ -71048,7 +72930,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>77</v>
       </c>
@@ -71059,7 +72941,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>78</v>
       </c>
@@ -71076,7 +72958,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>265</v>
       </c>
@@ -71084,7 +72966,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>79</v>
       </c>
@@ -71092,7 +72974,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>80</v>
       </c>
@@ -71103,7 +72985,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>81</v>
       </c>
@@ -71123,7 +73005,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>266</v>
       </c>
@@ -71131,7 +73013,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>82</v>
       </c>
@@ -71148,7 +73030,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>83</v>
       </c>
@@ -71176,8 +73058,11 @@
       <c r="J108" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K108" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>84</v>
       </c>
@@ -71194,7 +73079,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>85</v>
       </c>
@@ -71222,8 +73107,11 @@
       <c r="J110" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K110" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>86</v>
       </c>
@@ -71252,12 +73140,12 @@
         <v>86</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>87</v>
       </c>
@@ -71286,7 +73174,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>248</v>
       </c>
@@ -71294,7 +73182,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>88</v>
       </c>
@@ -71322,8 +73210,11 @@
       <c r="J115" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K115" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>89</v>
       </c>
@@ -71337,7 +73228,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>90</v>
       </c>
@@ -71351,7 +73242,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>91</v>
       </c>
@@ -71368,7 +73259,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>92</v>
       </c>
@@ -71385,7 +73276,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>93</v>
       </c>
@@ -71413,11 +73304,14 @@
       <c r="J120" t="s">
         <v>93</v>
       </c>
-      <c r="M120" t="s">
+      <c r="K120" t="s">
+        <v>305</v>
+      </c>
+      <c r="O120" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>94</v>
       </c>
@@ -71434,12 +73328,12 @@
         <v>94</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>95</v>
       </c>
@@ -71456,7 +73350,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>96</v>
       </c>
@@ -71485,7 +73379,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>97</v>
       </c>
@@ -71505,7 +73399,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>98</v>
       </c>
@@ -71519,7 +73413,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>99</v>
       </c>
@@ -71536,7 +73430,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>100</v>
       </c>
@@ -71556,7 +73450,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>101</v>
       </c>
@@ -71564,7 +73458,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>102</v>
       </c>
@@ -71572,7 +73466,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>103</v>
       </c>
@@ -71601,7 +73495,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>104</v>
       </c>
@@ -71618,7 +73512,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>105</v>
       </c>
@@ -71638,7 +73532,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>106</v>
       </c>
@@ -71652,7 +73546,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>107</v>
       </c>
@@ -71666,7 +73560,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>108</v>
       </c>
@@ -71680,7 +73574,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>109</v>
       </c>
@@ -71691,7 +73585,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>110</v>
       </c>
@@ -71702,7 +73596,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>111</v>
       </c>
@@ -71719,7 +73613,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>112</v>
       </c>
@@ -71730,7 +73624,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>113</v>
       </c>
@@ -71758,8 +73652,11 @@
       <c r="J141" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K141" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>114</v>
       </c>
@@ -71787,8 +73684,11 @@
       <c r="J142" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K142" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>115</v>
       </c>
@@ -71816,8 +73716,11 @@
       <c r="J143" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K143" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>116</v>
       </c>
@@ -71828,12 +73731,12 @@
         <v>116</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>117</v>
       </c>
@@ -71850,7 +73753,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>118</v>
       </c>
@@ -71861,7 +73764,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>119</v>
       </c>
@@ -71875,7 +73778,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>120</v>
       </c>
@@ -71892,7 +73795,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>121</v>
       </c>
@@ -71906,7 +73809,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>122</v>
       </c>
@@ -71938,7 +73841,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>123</v>
       </c>
@@ -71946,7 +73849,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>124</v>
       </c>
@@ -71965,8 +73868,11 @@
       <c r="J153" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K153" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>125</v>
       </c>
@@ -71980,7 +73886,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>126</v>
       </c>
@@ -72008,8 +73914,11 @@
       <c r="J155" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K155" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>127</v>
       </c>
@@ -72026,7 +73935,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>128</v>
       </c>
@@ -72039,8 +73948,11 @@
       <c r="J157" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K157" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>129</v>
       </c>
@@ -72057,7 +73969,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>130</v>
       </c>
@@ -72065,7 +73977,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>131</v>
       </c>
@@ -72079,7 +73991,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>132</v>
       </c>
@@ -72093,7 +74005,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>267</v>
       </c>
@@ -72101,7 +74013,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>268</v>
       </c>
@@ -72109,7 +74021,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>133</v>
       </c>
@@ -72120,7 +74032,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>134</v>
       </c>
@@ -72134,7 +74046,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>135</v>
       </c>
@@ -72154,7 +74066,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>269</v>
       </c>
@@ -72162,7 +74074,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>136</v>
       </c>
@@ -72176,7 +74088,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>137</v>
       </c>
@@ -72187,7 +74099,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>138</v>
       </c>
@@ -72201,7 +74113,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>270</v>
       </c>
@@ -72209,7 +74121,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>139</v>
       </c>
@@ -72226,7 +74138,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>140</v>
       </c>
@@ -72243,7 +74155,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>271</v>
       </c>
@@ -72251,7 +74163,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>141</v>
       </c>
@@ -72279,8 +74191,11 @@
       <c r="J175" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K175" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>142</v>
       </c>
@@ -72308,8 +74223,11 @@
       <c r="J176" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K176" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>143</v>
       </c>
@@ -72326,7 +74244,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>144</v>
       </c>
@@ -72334,7 +74252,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>145</v>
       </c>
@@ -72354,7 +74272,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>146</v>
       </c>
@@ -72368,7 +74286,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>147</v>
       </c>
@@ -72388,7 +74306,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>148</v>
       </c>
@@ -72405,7 +74323,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>272</v>
       </c>
@@ -72413,7 +74331,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>149</v>
       </c>
@@ -72436,7 +74354,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>150</v>
       </c>
@@ -72456,7 +74374,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>151</v>
       </c>
@@ -72464,7 +74382,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>152</v>
       </c>
@@ -72478,7 +74396,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>153</v>
       </c>
@@ -72506,8 +74424,11 @@
       <c r="J188" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K188" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>154</v>
       </c>
@@ -72515,7 +74436,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>155</v>
       </c>
@@ -72529,7 +74450,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>156</v>
       </c>
@@ -72557,8 +74478,11 @@
       <c r="J191" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K191" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>157</v>
       </c>
@@ -72578,7 +74502,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>158</v>
       </c>
@@ -72592,7 +74516,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>159</v>
       </c>
@@ -72603,7 +74527,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>160</v>
       </c>
@@ -72617,7 +74541,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>273</v>
       </c>
@@ -72625,7 +74549,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>161</v>
       </c>
@@ -72653,8 +74577,11 @@
       <c r="J197" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K197" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="198" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>162</v>
       </c>
@@ -72683,7 +74610,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>163</v>
       </c>
@@ -72697,7 +74624,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>164</v>
       </c>
@@ -72720,7 +74647,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>165</v>
       </c>
@@ -72731,7 +74658,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>166</v>
       </c>
@@ -72748,7 +74675,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>167</v>
       </c>
@@ -72768,7 +74695,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>276</v>
       </c>
@@ -72776,7 +74703,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>274</v>
       </c>
@@ -72784,7 +74711,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>277</v>
       </c>
@@ -72792,7 +74719,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>168</v>
       </c>
@@ -72800,7 +74727,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>169</v>
       </c>
@@ -72814,7 +74741,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>170</v>
       </c>
@@ -72831,7 +74758,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>171</v>
       </c>
@@ -72842,7 +74769,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>172</v>
       </c>
@@ -72856,7 +74783,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>278</v>
       </c>
@@ -72864,7 +74791,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>173</v>
       </c>
@@ -72884,7 +74811,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>174</v>
       </c>
@@ -72898,7 +74825,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>175</v>
       </c>
@@ -72912,7 +74839,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>442</v>
       </c>
@@ -72920,7 +74847,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>176</v>
       </c>
@@ -72934,7 +74861,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>177</v>
       </c>
@@ -72962,8 +74889,11 @@
       <c r="J218" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K218" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="219" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>178</v>
       </c>
@@ -72991,8 +74921,11 @@
       <c r="J219" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K219" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="220" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>179</v>
       </c>
@@ -73020,8 +74953,11 @@
       <c r="J220" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K220" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="221" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>180</v>
       </c>
@@ -73032,7 +74968,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>181</v>
       </c>
@@ -73040,7 +74976,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>182</v>
       </c>
@@ -73051,7 +74987,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>183</v>
       </c>
@@ -73065,7 +75001,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>184</v>
       </c>
@@ -73073,7 +75009,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>185</v>
       </c>
@@ -73087,7 +75023,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>186</v>
       </c>
@@ -73101,7 +75037,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>187</v>
       </c>
@@ -73121,7 +75057,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>188</v>
       </c>
@@ -73141,7 +75077,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>279</v>
       </c>
@@ -73149,7 +75085,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>189</v>
       </c>
@@ -73163,7 +75099,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>444</v>
       </c>
@@ -73171,7 +75107,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>190</v>
       </c>
@@ -73179,7 +75115,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>191</v>
       </c>
@@ -73190,7 +75126,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>192</v>
       </c>
@@ -73207,7 +75143,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>193</v>
       </c>
@@ -73235,8 +75171,11 @@
       <c r="J236" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K236" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="237" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>194</v>
       </c>
@@ -73244,7 +75183,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>195</v>
       </c>
@@ -73267,7 +75206,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>196</v>
       </c>
@@ -73281,7 +75220,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>197</v>
       </c>
@@ -73295,7 +75234,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="241" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>198</v>
       </c>
@@ -73312,7 +75251,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="242" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>281</v>
       </c>
@@ -73320,7 +75259,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="243" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>199</v>
       </c>
@@ -73340,7 +75279,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="244" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>200</v>
       </c>
@@ -73365,11 +75304,11 @@
       <c r="J244" t="s">
         <v>200</v>
       </c>
-      <c r="K244" t="s">
+      <c r="L244" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="245" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>201</v>
       </c>
@@ -73386,7 +75325,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="246" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>282</v>
       </c>
@@ -73394,7 +75333,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="247" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>202</v>
       </c>
@@ -73402,7 +75341,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="248" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>203</v>
       </c>
@@ -73422,7 +75361,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="249" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>204</v>
       </c>
@@ -73433,7 +75372,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="250" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>205</v>
       </c>
@@ -73441,7 +75380,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="251" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>206</v>
       </c>
@@ -73461,7 +75400,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="252" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>207</v>
       </c>
@@ -73472,7 +75411,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="253" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>283</v>
       </c>
@@ -73480,7 +75419,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="254" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>208</v>
       </c>
@@ -73491,12 +75430,15 @@
         <v>208</v>
       </c>
     </row>
-    <row r="255" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>440</v>
       </c>
-    </row>
-    <row r="256" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K255" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="256" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>209</v>
       </c>
@@ -73565,7 +75507,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:L259" xr:uid="{04039038-B78D-F44F-9F75-C547258D839A}"/>
+  <autoFilter ref="A2:N259" xr:uid="{04039038-B78D-F44F-9F75-C547258D839A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add BEA supply-use parser and docs
</commit_message>
<xml_diff>
--- a/doc/source/_static/data/Country_coverage.xlsx
+++ b/doc/source/_static/data/Country_coverage.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Documents/GitHub/MARIO/doc/source/_static/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45A92064-5E34-A543-B306-B24FE657FA07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496BAF02-A581-484A-830C-129D725F1C4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17660" activeTab="1" xr2:uid="{111A99A5-59A2-464B-993C-8B91581EF7C3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17660" xr2:uid="{111A99A5-59A2-464B-993C-8B91581EF7C3}"/>
   </bookViews>
   <sheets>
     <sheet name="coverage" sheetId="1" r:id="rId1"/>
     <sheet name="concordance" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">concordance!$A$2:$N$259</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">concordance!$A$2:$O$259</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23192" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23200" uniqueCount="500">
   <si>
     <t>ABW</t>
   </si>
@@ -1532,6 +1532,15 @@
   <si>
     <t>2018, 2020</t>
   </si>
+  <si>
+    <t>BEA</t>
+  </si>
+  <si>
+    <t>parse_bea</t>
+  </si>
+  <si>
+    <t>1997-2024</t>
+  </si>
 </sst>
 </file>
 
@@ -1945,7 +1954,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{637C923A-C55A-2E43-A14B-2765261D910F}">
-  <dimension ref="A1:IR948"/>
+  <dimension ref="A1:IR949"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -71211,6 +71220,26 @@
         <v>35</v>
       </c>
     </row>
+    <row r="949" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A949" t="s">
+        <v>497</v>
+      </c>
+      <c r="B949" t="s">
+        <v>498</v>
+      </c>
+      <c r="C949" t="s">
+        <v>344</v>
+      </c>
+      <c r="D949" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="G949" t="s">
+        <v>289</v>
+      </c>
+      <c r="H949" t="s">
+        <v>200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -71218,7 +71247,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04039038-B78D-F44F-9F75-C547258D839A}">
-  <dimension ref="A1:O259"/>
+  <dimension ref="A1:P259"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -71226,12 +71255,12 @@
     <col min="11" max="11" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>447</v>
       </c>
@@ -71269,16 +71298,19 @@
         <v>417</v>
       </c>
       <c r="M2" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -71296,7 +71328,7 @@
       </c>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -71316,7 +71348,7 @@
       </c>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -71338,7 +71370,7 @@
       </c>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>252</v>
       </c>
@@ -71351,7 +71383,7 @@
       <c r="H6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>434</v>
       </c>
@@ -71361,7 +71393,7 @@
       <c r="H7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -71388,7 +71420,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -71404,7 +71436,7 @@
       </c>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>253</v>
       </c>
@@ -71420,7 +71452,7 @@
       </c>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -71444,7 +71476,7 @@
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -71473,7 +71505,7 @@
       </c>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -71494,7 +71526,7 @@
       </c>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -71507,7 +71539,7 @@
       <c r="H14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>255</v>
       </c>
@@ -71520,7 +71552,7 @@
       <c r="H15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>256</v>
       </c>
@@ -71815,7 +71847,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>22</v>
       </c>
@@ -71832,7 +71864,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -71846,7 +71878,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>24</v>
       </c>
@@ -71857,7 +71889,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -71877,7 +71909,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>26</v>
       </c>
@@ -71909,7 +71941,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -71920,7 +71952,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>28</v>
       </c>
@@ -71940,7 +71972,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>29</v>
       </c>
@@ -71957,7 +71989,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>258</v>
       </c>
@@ -71965,7 +71997,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>30</v>
       </c>
@@ -71979,7 +72011,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>31</v>
       </c>
@@ -71993,7 +72025,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>32</v>
       </c>
@@ -72021,11 +72053,11 @@
       <c r="J44" t="s">
         <v>32</v>
       </c>
-      <c r="N44" t="s">
+      <c r="O44" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>259</v>
       </c>
@@ -72033,7 +72065,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>33</v>
       </c>
@@ -72062,12 +72094,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>34</v>
       </c>
@@ -72090,7 +72122,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>35</v>
       </c>
@@ -72118,11 +72150,11 @@
       <c r="J49" t="s">
         <v>35</v>
       </c>
-      <c r="M49" t="s">
+      <c r="N49" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>36</v>
       </c>
@@ -72139,7 +72171,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>37</v>
       </c>
@@ -72156,7 +72188,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>38</v>
       </c>
@@ -72173,7 +72205,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>39</v>
       </c>
@@ -72187,7 +72219,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>260</v>
       </c>
@@ -72195,7 +72227,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>40</v>
       </c>
@@ -72218,7 +72250,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>41</v>
       </c>
@@ -72226,7 +72258,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>42</v>
       </c>
@@ -72240,7 +72272,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>43</v>
       </c>
@@ -72260,7 +72292,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>44</v>
       </c>
@@ -72274,7 +72306,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>45</v>
       </c>
@@ -72282,7 +72314,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>261</v>
       </c>
@@ -72290,7 +72322,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>46</v>
       </c>
@@ -72301,7 +72333,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>47</v>
       </c>
@@ -72333,7 +72365,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>48</v>
       </c>
@@ -73145,7 +73177,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>87</v>
       </c>
@@ -73174,7 +73206,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>248</v>
       </c>
@@ -73182,7 +73214,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>88</v>
       </c>
@@ -73214,7 +73246,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>89</v>
       </c>
@@ -73228,7 +73260,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>90</v>
       </c>
@@ -73242,7 +73274,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>91</v>
       </c>
@@ -73259,7 +73291,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>92</v>
       </c>
@@ -73276,7 +73308,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>93</v>
       </c>
@@ -73307,11 +73339,11 @@
       <c r="K120" t="s">
         <v>305</v>
       </c>
-      <c r="O120" t="s">
+      <c r="P120" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>94</v>
       </c>
@@ -73328,12 +73360,12 @@
         <v>94</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>95</v>
       </c>
@@ -73350,7 +73382,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>96</v>
       </c>
@@ -73379,7 +73411,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>97</v>
       </c>
@@ -73399,7 +73431,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>98</v>
       </c>
@@ -73413,7 +73445,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>99</v>
       </c>
@@ -73430,7 +73462,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>100</v>
       </c>
@@ -75234,7 +75266,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>198</v>
       </c>
@@ -75251,7 +75283,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>281</v>
       </c>
@@ -75259,7 +75291,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>199</v>
       </c>
@@ -75279,7 +75311,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>200</v>
       </c>
@@ -75307,8 +75339,11 @@
       <c r="L244" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M244" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="245" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>201</v>
       </c>
@@ -75325,7 +75360,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>282</v>
       </c>
@@ -75333,7 +75368,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>202</v>
       </c>
@@ -75341,7 +75376,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>203</v>
       </c>
@@ -75361,7 +75396,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>204</v>
       </c>
@@ -75372,7 +75407,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>205</v>
       </c>
@@ -75380,7 +75415,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>206</v>
       </c>
@@ -75400,7 +75435,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>207</v>
       </c>
@@ -75411,7 +75446,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>283</v>
       </c>
@@ -75419,7 +75454,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>208</v>
       </c>
@@ -75430,7 +75465,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>440</v>
       </c>
@@ -75438,7 +75473,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>209</v>
       </c>
@@ -75507,7 +75542,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:N259" xr:uid="{04039038-B78D-F44F-9F75-C547258D839A}"/>
+  <autoFilter ref="A2:O259" xr:uid="{04039038-B78D-F44F-9F75-C547258D839A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>